<commit_message>
auto commit: 2026-03-20 09:57:55
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -219,8 +219,14 @@
       <color rgb="00C00000"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="000D47A1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -431,8 +437,20 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D47A1"/>
+        <bgColor rgb="000D47A1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -566,6 +584,50 @@
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
@@ -715,7 +777,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -750,6 +812,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1199,7 +1270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J580"/>
+  <dimension ref="A1:J627"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="6.5" customWidth="1" style="3" min="1" max="3"/>
@@ -20057,7 +20128,6 @@
       </c>
       <c r="J453" s="4" t="inlineStr"/>
     </row>
-    <row r="454"/>
     <row r="455">
       <c r="A455" s="7" t="inlineStr">
         <is>
@@ -24678,7 +24748,6 @@
         </is>
       </c>
     </row>
-    <row r="550"/>
     <row r="551">
       <c r="A551" s="13" t="inlineStr">
         <is>
@@ -24692,59 +24761,15 @@
           <t>用户端</t>
         </is>
       </c>
-      <c r="B552" s="9" t="inlineStr">
-        <is>
-          <t>1.5h</t>
-        </is>
-      </c>
-      <c r="C552" s="9" t="inlineStr">
-        <is>
-          <t>xcx-sm-001</t>
-        </is>
-      </c>
-      <c r="D552" s="9" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E552" s="9" t="inlineStr">
-        <is>
-          <t>小程序环境
-(生命周期/启动)</t>
-        </is>
-      </c>
-      <c r="F552" s="9" t="inlineStr">
-        <is>
-          <t>验证小程序冷启动正常加载</t>
-        </is>
-      </c>
-      <c r="G552" s="9" t="inlineStr">
-        <is>
-          <t>1. 小程序未在微信后台运行
-2. 用户已有微信登录态</t>
-        </is>
-      </c>
-      <c r="H552" s="9" t="inlineStr">
-        <is>
-          <t>1. 在微信中搜索或扫码打开快乐羊毛小程序。
-2. 观察启动过程（闪屏/loading）。
-3. 记录从点击到首页完全渲染的时间。
-4. 检查首页数据是否完整加载</t>
-        </is>
-      </c>
-      <c r="I552" s="9" t="inlineStr">
-        <is>
-          <t>1. 启动过程有品牌闪屏（如有配置）。
-2. 首屏渲染&lt;2秒（WiFi）/&lt;5秒（4G）。
-3. 首页数据完整加载，不出现白屏。
-4. 用户登录态自动恢复（微信静默登录）</t>
-        </is>
-      </c>
-      <c r="J552" s="9" t="inlineStr">
-        <is>
-          <t>冷启动是用户最常遇到的入口场景</t>
-        </is>
-      </c>
+      <c r="B552" s="16" t="n"/>
+      <c r="C552" s="16" t="n"/>
+      <c r="D552" s="16" t="n"/>
+      <c r="E552" s="16" t="n"/>
+      <c r="F552" s="16" t="n"/>
+      <c r="G552" s="16" t="n"/>
+      <c r="H552" s="16" t="n"/>
+      <c r="I552" s="16" t="n"/>
+      <c r="J552" s="17" t="n"/>
     </row>
     <row r="553">
       <c r="A553" s="8" t="inlineStr"/>
@@ -26159,13 +26184,2378 @@
         </is>
       </c>
     </row>
+    <row r="582">
+      <c r="A582" s="18" t="inlineStr">
+        <is>
+          <t>═══ 各功能模块 · 小程序环境专项用例 ═══ 每个模块在微信小程序中的具体操作行为、交互、异常 ═══</t>
+        </is>
+      </c>
+      <c r="B582" s="19" t="n"/>
+      <c r="C582" s="19" t="n"/>
+      <c r="D582" s="19" t="n"/>
+      <c r="E582" s="19" t="n"/>
+      <c r="F582" s="19" t="n"/>
+      <c r="G582" s="19" t="n"/>
+      <c r="H582" s="19" t="n"/>
+      <c r="I582" s="19" t="n"/>
+      <c r="J582" s="19" t="n"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B583" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C583" s="20" t="inlineStr">
+        <is>
+          <t>mfzl-xcx-001</t>
+        </is>
+      </c>
+      <c r="D583" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E583" s="20" t="inlineStr">
+        <is>
+          <t>免费资料区
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F583" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序内复制链接调用剪贴板后的微信原生Toast提示</t>
+        </is>
+      </c>
+      <c r="G583" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户已进入免费资料区详情页
+2. 详情页有可复制链接</t>
+        </is>
+      </c>
+      <c r="H583" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击"复制链接"按钮。
+2. 观察弹出的Toast提示样式。
+3. 长按微信聊天输入框粘贴，验证剪贴板内容正确。
+4. 等待Toast消失（约2秒）</t>
+        </is>
+      </c>
+      <c r="I583" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击后弹出"复制成功"Toast（微信原生样式，非自定义弹窗）。
+2. Toast约2秒后自动消失。
+3. 粘贴内容为完整链接URL。
+4. 不弹出微信"是否允许读取剪贴板"授权提示（写入不需要）</t>
+        </is>
+      </c>
+      <c r="J583" s="20" t="inlineStr">
+        <is>
+          <t>小程序调用wx.setClipboardData会弹微信原生Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="8" t="inlineStr"/>
+      <c r="B584" s="8" t="inlineStr"/>
+      <c r="C584" s="8" t="inlineStr">
+        <is>
+          <t>mfzl-xcx-002</t>
+        </is>
+      </c>
+      <c r="D584" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E584" s="8" t="n"/>
+      <c r="F584" s="8" t="inlineStr">
+        <is>
+          <t>验证资料列表页小程序下拉刷新和触底加载交互</t>
+        </is>
+      </c>
+      <c r="G584" s="8" t="inlineStr">
+        <is>
+          <t>1. 免费资料区已有20+条数据
+2. 小程序已开启enablePullDownRefresh</t>
+        </is>
+      </c>
+      <c r="H584" s="8" t="inlineStr">
+        <is>
+          <t>1. 在列表页顶部下拉。
+2. 观察下拉刷新动画（微信原生三个点）。
+3. 松手后数据刷新。
+4. 滚动到列表底部。
+5. 观察触底加载更多行为</t>
+        </is>
+      </c>
+      <c r="I584" s="8" t="inlineStr">
+        <is>
+          <t>1. 下拉显示微信原生刷新动画（绿色三个点）。
+2. 松手后触发onPullDownRefresh，数据刷新，动画结束。
+3. 触底自动触发onReachBottom加载下一页。
+4. 加载中显示"加载中..."。
+5. 最后一页显示"没有更多了"</t>
+        </is>
+      </c>
+      <c r="J584" s="8" t="inlineStr">
+        <is>
+          <t>小程序下拉刷新是原生Page事件，非自定义组件</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="8" t="inlineStr"/>
+      <c r="B585" s="8" t="inlineStr"/>
+      <c r="C585" s="8" t="inlineStr">
+        <is>
+          <t>mfzl-xcx-003</t>
+        </is>
+      </c>
+      <c r="D585" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E585" s="8" t="n"/>
+      <c r="F585" s="8" t="inlineStr">
+        <is>
+          <t>验证详情页返回列表时页面栈保持和滚动位置恢复</t>
+        </is>
+      </c>
+      <c r="G585" s="8" t="inlineStr">
+        <is>
+          <t>1. 列表已滚动到第15条数据位置
+2. 准备点击某条进入详情</t>
+        </is>
+      </c>
+      <c r="H585" s="8" t="inlineStr">
+        <is>
+          <t>1. 记录当前滚动位置（约第15条）。
+2. 点击某条资料进入详情页（navigateTo压栈）。
+3. 点击左上角返回按钮（navigateBack出栈）。
+4. 检查列表页状态</t>
+        </is>
+      </c>
+      <c r="I585" s="8" t="inlineStr">
+        <is>
+          <t>1. 进入详情页时列表页保留在页面栈中。
+2. 返回后列表恢复到第15条位置，不回到顶部。
+3. 已加载的数据不丢失、不重复请求。
+4. 页面栈深度不超过10层（小程序限制）</t>
+        </is>
+      </c>
+      <c r="J585" s="8" t="inlineStr">
+        <is>
+          <t>小程序navigateTo最大10层页面栈</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="8" t="inlineStr"/>
+      <c r="B586" s="8" t="inlineStr"/>
+      <c r="C586" s="8" t="inlineStr">
+        <is>
+          <t>mfzl-xcx-004</t>
+        </is>
+      </c>
+      <c r="D586" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E586" s="8" t="n"/>
+      <c r="F586" s="8" t="inlineStr">
+        <is>
+          <t>验证资料区转发分享给好友后对方能正确打开</t>
+        </is>
+      </c>
+      <c r="G586" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户在免费资料详情页</t>
+        </is>
+      </c>
+      <c r="H586" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击右上角"..."胶囊按钮。
+2. 选择"转发"。
+3. 选择好友发送。
+4. 好友在聊天中点击分享卡片</t>
+        </is>
+      </c>
+      <c r="I586" s="8" t="inlineStr">
+        <is>
+          <t>1. 分享卡片显示资料标题和描述。
+2. 好友点击后直接进入该资料详情页（非首页）。
+3. 详情页数据正确加载。
+4. 好友可正常返回首页浏览其他内容</t>
+        </is>
+      </c>
+      <c r="J586" s="8" t="inlineStr">
+        <is>
+          <t>小程序分享需配置onShareAppMessage</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B587" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C587" s="20" t="inlineStr">
+        <is>
+          <t>wamhb-xcx-001</t>
+        </is>
+      </c>
+      <c r="D587" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E587" s="20" t="inlineStr">
+        <is>
+          <t>外卖区-红包
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F587" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序内跳转外部App（美团/饿了么）的行为</t>
+        </is>
+      </c>
+      <c r="G587" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户在外卖红包页面
+2. 手机已安装美团App</t>
+        </is>
+      </c>
+      <c r="H587" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击美团红包Icon。
+2. 中间页加载完成。
+3. 观察跳转行为（小程序→App）。
+4. 从美团App返回小程序</t>
+        </is>
+      </c>
+      <c r="I587" s="20" t="inlineStr">
+        <is>
+          <t>1. 小程序通过scheme/universal link唤起美团App。
+2. 跳转时微信可能弹出"即将打开外部应用"确认框。
+3. 确认后成功打开美团对应页面。
+4. 从美团App返回微信后，小程序热启动恢复到红包页面</t>
+        </is>
+      </c>
+      <c r="J587" s="20" t="inlineStr">
+        <is>
+          <t>小程序跳转外部App需要配置URL Scheme白名单</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="8" t="inlineStr"/>
+      <c r="B588" s="8" t="inlineStr"/>
+      <c r="C588" s="8" t="inlineStr">
+        <is>
+          <t>wamhb-xcx-002</t>
+        </is>
+      </c>
+      <c r="D588" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E588" s="8" t="n"/>
+      <c r="F588" s="8" t="inlineStr">
+        <is>
+          <t>验证手机未安装目标App时小程序降级为H5内嵌打开</t>
+        </is>
+      </c>
+      <c r="G588" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户手机未安装饿了么App</t>
+        </is>
+      </c>
+      <c r="H588" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击饿了么红包Icon。
+2. 观察跳转行为</t>
+        </is>
+      </c>
+      <c r="I588" s="8" t="inlineStr">
+        <is>
+          <t>1. 检测到未安装App，不尝试唤起。
+2. 在小程序内嵌web-view中打开H5页面。
+3. 或弹出提示"未安装饿了么App，是否下载？"。
+4. H5页面正常显示领券内容</t>
+        </is>
+      </c>
+      <c r="J588" s="8" t="inlineStr">
+        <is>
+          <t>小程序需判断canLaunch再决定跳转方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="8" t="inlineStr"/>
+      <c r="B589" s="8" t="inlineStr"/>
+      <c r="C589" s="8" t="inlineStr">
+        <is>
+          <t>wamhb-xcx-003</t>
+        </is>
+      </c>
+      <c r="D589" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E589" s="8" t="n"/>
+      <c r="F589" s="8" t="inlineStr">
+        <is>
+          <t>验证外卖红包页面小程序分享卡片内容正确</t>
+        </is>
+      </c>
+      <c r="G589" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户在外卖红包页面</t>
+        </is>
+      </c>
+      <c r="H589" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击右上角"..."。
+2. 选择"转发"给好友。
+3. 好友收到后点击分享卡片</t>
+        </is>
+      </c>
+      <c r="I589" s="8" t="inlineStr">
+        <is>
+          <t>1. 分享卡片标题如"快乐羊毛·外卖红包"。
+2. 卡片封面图正确。
+3. 好友点击后进入外卖红包页面（含推广参数）。
+4. 推广关系正确绑定</t>
+        </is>
+      </c>
+      <c r="J589" s="8" t="inlineStr">
+        <is>
+          <t>分享卡片是用户裂变的核心渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B590" s="20" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="C590" s="20" t="inlineStr">
+        <is>
+          <t>wamtyj-xcx-001</t>
+        </is>
+      </c>
+      <c r="D590" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E590" s="20" t="inlineStr">
+        <is>
+          <t>外卖区-通用券
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F590" s="20" t="inlineStr">
+        <is>
+          <t>验证通用券购买全流程在小程序中的微信支付交互</t>
+        </is>
+      </c>
+      <c r="G590" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户已选择10元面额通用券
+2. 确认订单页已展示</t>
+        </is>
+      </c>
+      <c r="H590" s="20" t="inlineStr">
+        <is>
+          <t>1. 确认红色"支付后不退款"提示文案可见。
+2. 勾选"已阅读并同意"协议复选框。
+3. 点击"确认支付"。
+4. 微信支付弹窗从底部弹出。
+5. 确认弹窗显示金额（如¥9.50）和收款方。
+6. 输入6位支付密码。
+7. 支付完成后观察页面跳转</t>
+        </is>
+      </c>
+      <c r="I590" s="20" t="inlineStr">
+        <is>
+          <t>1. 微信支付弹窗正常唤起（wx.requestPayment）。
+2. 弹窗显示正确金额和"快乐羊毛"收款方。
+3. 输入密码后弹窗消失，返回小程序。
+4. 自动跳转到订单结果页展示卡密。
+5. 整个过程不超过3秒</t>
+        </is>
+      </c>
+      <c r="J590" s="20" t="inlineStr">
+        <is>
+          <t>小程序支付通过wx.requestPayment调起</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="8" t="inlineStr"/>
+      <c r="B591" s="8" t="inlineStr"/>
+      <c r="C591" s="8" t="inlineStr">
+        <is>
+          <t>wamtyj-xcx-002</t>
+        </is>
+      </c>
+      <c r="D591" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E591" s="8" t="n"/>
+      <c r="F591" s="8" t="inlineStr">
+        <is>
+          <t>验证小程序支付弹窗取消后可重新发起支付</t>
+        </is>
+      </c>
+      <c r="G591" s="8" t="inlineStr">
+        <is>
+          <t>1. 支付弹窗已唤起</t>
+        </is>
+      </c>
+      <c r="H591" s="8" t="inlineStr">
+        <is>
+          <t>1. 在支付弹窗上点击右上角"×"关闭。
+2. 返回到订单确认页。
+3. 检查页面状态和按钮可用性。
+4. 再次点击"确认支付"</t>
+        </is>
+      </c>
+      <c r="I591" s="8" t="inlineStr">
+        <is>
+          <t>1. 关闭弹窗后小程序收到fail回调（errMsg: requestPayment:fail cancel）。
+2. 订单状态保持"待支付"。
+3. 支付按钮恢复可点击。
+4. 再次点击正常唤起支付弹窗。
+5. 不产生重复订单</t>
+        </is>
+      </c>
+      <c r="J591" s="8" t="inlineStr">
+        <is>
+          <t>用户可能反复取消再支付</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="8" t="inlineStr"/>
+      <c r="B592" s="8" t="inlineStr"/>
+      <c r="C592" s="8" t="inlineStr">
+        <is>
+          <t>wamtyj-xcx-003</t>
+        </is>
+      </c>
+      <c r="D592" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E592" s="8" t="n"/>
+      <c r="F592" s="8" t="inlineStr">
+        <is>
+          <t>验证卡密复制按钮在小程序中的剪贴板行为</t>
+        </is>
+      </c>
+      <c r="G592" s="8" t="inlineStr">
+        <is>
+          <t>1. 通用券购买成功
+2. 订单详情展示卡密信息</t>
+        </is>
+      </c>
+      <c r="H592" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击"复制卡密"按钮。
+2. 观察提示。
+3. 切换到微信聊天窗口粘贴验证。
+4. 返回小程序点击"复制券码"</t>
+        </is>
+      </c>
+      <c r="I592" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击后微信弹出原生"内容已复制"Toast。
+2. 粘贴内容为完整卡密号。
+3. 切换回小程序页面不丢失数据。
+4. 券码复制同样正常</t>
+        </is>
+      </c>
+      <c r="J592" s="8" t="inlineStr">
+        <is>
+          <t>小程序复制后自动弹微信系统Toast</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="8" t="inlineStr"/>
+      <c r="B593" s="8" t="inlineStr"/>
+      <c r="C593" s="8" t="inlineStr">
+        <is>
+          <t>wamtyj-xcx-004</t>
+        </is>
+      </c>
+      <c r="D593" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E593" s="8" t="n"/>
+      <c r="F593" s="8" t="inlineStr">
+        <is>
+          <t>验证通用券下单确认页"不退款"协议勾选框的小程序交互</t>
+        </is>
+      </c>
+      <c r="G593" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已选择面额，进入确认页</t>
+        </is>
+      </c>
+      <c r="H593" s="8" t="inlineStr">
+        <is>
+          <t>1. 不勾选协议，直接点击"确认支付"。
+2. 观察按钮状态和提示。
+3. 勾选协议复选框。
+4. 再次点击"确认支付"</t>
+        </is>
+      </c>
+      <c r="I593" s="8" t="inlineStr">
+        <is>
+          <t>1. 未勾选时：支付按钮为灰色不可点击，或点击后提示"请先勾选协议"。
+2. 勾选后：支付按钮变为可点击状态（颜色变化）。
+3. 点击后正常唤起微信支付弹窗</t>
+        </is>
+      </c>
+      <c r="J593" s="8" t="inlineStr">
+        <is>
+          <t>此勾选框是合规要求，必须拦截未勾选</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B594" s="20" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="C594" s="20" t="inlineStr">
+        <is>
+          <t>cyzkxtzl-xcx-001</t>
+        </is>
+      </c>
+      <c r="D594" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E594" s="20" t="inlineStr">
+        <is>
+          <t>餐饮折扣-系统直连
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F594" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序扫码支付全流程（wx.scanCode → 支付）</t>
+        </is>
+      </c>
+      <c r="G594" s="20" t="inlineStr">
+        <is>
+          <t>1. 商家已在小程序端生成收款二维码
+2. 用户打开快乐羊毛小程序</t>
+        </is>
+      </c>
+      <c r="H594" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户在小程序内点击"扫码支付"。
+2. 小程序调起摄像头（首次弹授权）。
+3. 对准商家二维码扫描。
+4. 扫码成功，跳转到支付确认页。
+5. 确认原价/优惠/实付金额。
+6. 点击支付，微信支付弹窗弹出。
+7. 输入密码完成支付</t>
+        </is>
+      </c>
+      <c r="I594" s="20" t="inlineStr">
+        <is>
+          <t>1. 扫码功能正常调起（wx.scanCode）。
+2. 首次使用弹出摄像头授权，允许后正常扫描。
+3. 扫码解析二维码内容并跳转正确页面。
+4. 支付确认页展示正确的金额（如原价100/优惠20/实付80）。
+5. 微信支付正常完成。
+6. 支付成功后跳转结果页，三端数据同步</t>
+        </is>
+      </c>
+      <c r="J594" s="20" t="inlineStr">
+        <is>
+          <t>扫码→解析→支付是小程序核心链路</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="8" t="inlineStr"/>
+      <c r="B595" s="8" t="inlineStr"/>
+      <c r="C595" s="8" t="inlineStr">
+        <is>
+          <t>cyzkxtzl-xcx-002</t>
+        </is>
+      </c>
+      <c r="D595" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E595" s="8" t="n"/>
+      <c r="F595" s="8" t="inlineStr">
+        <is>
+          <t>验证用户通过微信"扫一扫"扫商家码进入小程序支付</t>
+        </is>
+      </c>
+      <c r="G595" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家已生成收款二维码
+2. 用户在微信首页</t>
+        </is>
+      </c>
+      <c r="H595" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户在微信首页点击右上角"+"→"扫一扫"。
+2. 扫描商家收款二维码。
+3. 微信识别为小程序码后自动打开快乐羊毛小程序。
+4. 小程序直接跳转到支付确认页。
+5. 完成支付</t>
+        </is>
+      </c>
+      <c r="I595" s="8" t="inlineStr">
+        <is>
+          <t>1. 微信扫一扫正确识别二维码。
+2. 自动打开快乐羊毛小程序（冷启动或热启动）。
+3. 通过scene参数直接跳转到支付页面，不经过首页。
+4. 支付确认页展示正确金额。
+5. 支付流程正常完成</t>
+        </is>
+      </c>
+      <c r="J595" s="8" t="inlineStr">
+        <is>
+          <t>用户可能直接从微信扫一扫进入，不是从小程序内部扫码</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="8" t="inlineStr"/>
+      <c r="B596" s="8" t="inlineStr"/>
+      <c r="C596" s="8" t="inlineStr">
+        <is>
+          <t>cyzkxtzl-xcx-003</t>
+        </is>
+      </c>
+      <c r="D596" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E596" s="8" t="n"/>
+      <c r="F596" s="8" t="inlineStr">
+        <is>
+          <t>验证二维码生成后的小程序前后台切换不影响有效性</t>
+        </is>
+      </c>
+      <c r="G596" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家端小程序已生成收款二维码
+2. 二维码有15分钟倒计时</t>
+        </is>
+      </c>
+      <c r="H596" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家生成二维码后按Home键将小程序切到后台。
+2. 等待3分钟。
+3. 回到小程序前台。
+4. 检查二维码和倒计时状态。
+5. 让用户扫码支付</t>
+        </is>
+      </c>
+      <c r="I596" s="8" t="inlineStr">
+        <is>
+          <t>1. 切回前台后二维码仍然显示。
+2. 倒计时正确更新（从服务端同步时间而非本地计时）。
+3. 用户扫码支付正常完成。
+4. 如小程序被系统回收重启，重新加载收银台页面</t>
+        </is>
+      </c>
+      <c r="J596" s="8" t="inlineStr">
+        <is>
+          <t>商家经常切后台聊天再回来——二维码不能丢</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="8" t="inlineStr"/>
+      <c r="B597" s="8" t="inlineStr"/>
+      <c r="C597" s="8" t="inlineStr">
+        <is>
+          <t>cyzkxtzl-xcx-004</t>
+        </is>
+      </c>
+      <c r="D597" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E597" s="8" t="n"/>
+      <c r="F597" s="8" t="inlineStr">
+        <is>
+          <t>验证餐饮折扣收银台小程序数字键盘输入金额</t>
+        </is>
+      </c>
+      <c r="G597" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家端小程序已打开收银台页面</t>
+        </is>
+      </c>
+      <c r="H597" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击金额输入框。
+2. 观察弹出的键盘类型。
+3. 输入金额"99.50"。
+4. 点击输入框外收起键盘。
+5. 检查折扣自动计算</t>
+        </is>
+      </c>
+      <c r="I597" s="8" t="inlineStr">
+        <is>
+          <t>1. 弹出小程序数字键盘（type="digit"带小数点）。
+2. 键盘不遮挡金额和折扣展示区域（页面自动上推）。
+3. 输入99.50后实时计算折扣（如8折=79.60）。
+4. 收起键盘后金额保持。
+5. 计算结果正确显示</t>
+        </is>
+      </c>
+      <c r="J597" s="8" t="inlineStr">
+        <is>
+          <t>小程序input的type="digit"唤起带小数点的数字键盘</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B598" s="20" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="C598" s="20" t="inlineStr">
+        <is>
+          <t>cyzkrg-xcx-001</t>
+        </is>
+      </c>
+      <c r="D598" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E598" s="20" t="inlineStr">
+        <is>
+          <t>餐饮折扣-人工辅助
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F598" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序内拍照/相册选择上传凭证（wx.chooseImage）</t>
+        </is>
+      </c>
+      <c r="G598" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户在人工辅助模式下单页
+2. 已输入消费金额</t>
+        </is>
+      </c>
+      <c r="H598" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击"上传凭证"按钮。
+2. 小程序弹出ActionSheet："拍照"/"从相册选择"。
+3. 选择"拍照"，摄像头打开。
+4. 拍照后确认使用该照片。
+5. 再次点击上传，选择"从相册选择"。
+6. 从相册选择一张图片</t>
+        </is>
+      </c>
+      <c r="I598" s="20" t="inlineStr">
+        <is>
+          <t>1. ActionSheet正常弹出（wx.chooseMedia/wx.chooseImage）。
+2. 选择拍照后摄像头授权弹窗正常。
+3. 拍照后图片压缩上传，缩略图正确展示。
+4. 从相册选择后图片正常上传。
+5. 支持多次选择上传多张（最多5张）</t>
+        </is>
+      </c>
+      <c r="J598" s="20" t="inlineStr">
+        <is>
+          <t>小程序图片选择API在iOS和Android行为不同</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="8" t="inlineStr"/>
+      <c r="B599" s="8" t="inlineStr"/>
+      <c r="C599" s="8" t="inlineStr">
+        <is>
+          <t>cyzkrg-xcx-002</t>
+        </is>
+      </c>
+      <c r="D599" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E599" s="8" t="n"/>
+      <c r="F599" s="8" t="inlineStr">
+        <is>
+          <t>验证凭证图片预览大图（wx.previewImage）</t>
+        </is>
+      </c>
+      <c r="G599" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已上传2张凭证图片</t>
+        </is>
+      </c>
+      <c r="H599" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击第1张缩略图。
+2. 观察预览行为。
+3. 在预览中左右滑动。
+4. 点击返回关闭预览</t>
+        </is>
+      </c>
+      <c r="I599" s="8" t="inlineStr">
+        <is>
+          <t>1. 调用wx.previewImage打开微信原生图片预览。
+2. 图片全屏展示，支持双指缩放。
+3. 左右滑动可查看其他已上传图片。
+4. 点击返回回到上传页面，数据不丢失</t>
+        </is>
+      </c>
+      <c r="J599" s="8" t="inlineStr">
+        <is>
+          <t>小程序图片预览是微信原生全屏预览体验</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="8" t="inlineStr"/>
+      <c r="B600" s="8" t="inlineStr"/>
+      <c r="C600" s="8" t="inlineStr">
+        <is>
+          <t>cyzkrg-xcx-003</t>
+        </is>
+      </c>
+      <c r="D600" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E600" s="8" t="n"/>
+      <c r="F600" s="8" t="inlineStr">
+        <is>
+          <t>验证用户收到验证码的小程序订阅消息推送</t>
+        </is>
+      </c>
+      <c r="G600" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已授权订阅消息
+2. 运营已审核通过并输入验证码</t>
+        </is>
+      </c>
+      <c r="H600" s="8" t="inlineStr">
+        <is>
+          <t>1. 运营在后台点击"确认下发"验证码。
+2. 用户手机检查微信消息通知。
+3. 点击订阅消息卡片。
+4. 查看消息详情</t>
+        </is>
+      </c>
+      <c r="I600" s="8" t="inlineStr">
+        <is>
+          <t>1. 微信"服务通知"出现新消息（&lt;1分钟内）。
+2. 消息卡片显示：快乐羊毛发来服务通知。
+3. 点击卡片进入小程序订单详情页。
+4. 详情页展示验证码+商家名称+消费金额。
+5. 验证码可复制或展示给商家</t>
+        </is>
+      </c>
+      <c r="J600" s="8" t="inlineStr">
+        <is>
+          <t>订阅消息需要用户在小程序内主动授权触发</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="8" t="inlineStr"/>
+      <c r="B601" s="8" t="inlineStr"/>
+      <c r="C601" s="8" t="inlineStr">
+        <is>
+          <t>cyzkrg-xcx-004</t>
+        </is>
+      </c>
+      <c r="D601" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E601" s="8" t="n"/>
+      <c r="F601" s="8" t="inlineStr">
+        <is>
+          <t>验证用户未授权订阅消息时验证码的降级通知</t>
+        </is>
+      </c>
+      <c r="G601" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户拒绝了订阅消息授权
+2. 运营已下发验证码</t>
+        </is>
+      </c>
+      <c r="H601" s="8" t="inlineStr">
+        <is>
+          <t>1. 运营下发验证码。
+2. 系统检测到用户未授权订阅消息。
+3. 自动降级发送短信通知。
+4. 用户查看短信</t>
+        </is>
+      </c>
+      <c r="I601" s="8" t="inlineStr">
+        <is>
+          <t>1. 小程序订阅消息发送失败（用户未授权）。
+2. 系统自动降级为短信推送。
+3. 用户手机收到短信（含验证码/商家名/金额）。
+4. 同时，用户在小程序"我的订单"详情页也能查看验证码。
+5. 不因推送失败阻塞业务流程</t>
+        </is>
+      </c>
+      <c r="J601" s="8" t="inlineStr">
+        <is>
+          <t>三级降级：订阅消息→短信→订单详情页查看</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="8" t="inlineStr"/>
+      <c r="B602" s="8" t="inlineStr"/>
+      <c r="C602" s="8" t="inlineStr">
+        <is>
+          <t>cyzkrg-xcx-005</t>
+        </is>
+      </c>
+      <c r="D602" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E602" s="8" t="n"/>
+      <c r="F602" s="8" t="inlineStr">
+        <is>
+          <t>验证商家端小程序核销验证码的输入与确认交互</t>
+        </is>
+      </c>
+      <c r="G602" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家端小程序已登录
+2. 用户到店出示验证码</t>
+        </is>
+      </c>
+      <c r="H602" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家在小程序订单详情页点击"核销"。
+2. 弹出验证码输入弹窗/页面。
+3. 输入用户告知的验证码。
+4. 点击"确认核销"。
+5. 核销成功</t>
+        </is>
+      </c>
+      <c r="I602" s="8" t="inlineStr">
+        <is>
+          <t>1. 输入框获取焦点后弹出数字键盘。
+2. 输入验证码后按钮变为可点击。
+3. 点击核销后loading状态（防重复点击）。
+4. 核销成功弹出"核销成功"Toast。
+5. 订单状态实时更新为"已完成"</t>
+        </is>
+      </c>
+      <c r="J602" s="8" t="inlineStr">
+        <is>
+          <t>商家操作场景——简洁快速</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B603" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C603" s="20" t="inlineStr">
+        <is>
+          <t>dcfw-xcx-001</t>
+        </is>
+      </c>
+      <c r="D603" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E603" s="20" t="inlineStr">
+        <is>
+          <t>打车服务
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F603" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序获取位置权限（wx.getLocation）及定位</t>
+        </is>
+      </c>
+      <c r="G603" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户首次使用打车服务
+2. 手机GPS已开启</t>
+        </is>
+      </c>
+      <c r="H603" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击"打车服务"入口。
+2. 小程序弹出位置授权弹窗。
+3. 点击"允许"。
+4. 观察定位结果</t>
+        </is>
+      </c>
+      <c r="I603" s="20" t="inlineStr">
+        <is>
+          <t>1. 微信原生授权弹窗："快乐羊毛申请获取你的地理位置"。
+2. 允许后获取当前GPS坐标。
+3. 页面展示当前位置地址（逆地理编码）。
+4. 定位精度在可接受范围内（偏差&lt;100米）</t>
+        </is>
+      </c>
+      <c r="J603" s="20" t="inlineStr">
+        <is>
+          <t>小程序wx.getLocation需要在app.json配置permission</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="8" t="inlineStr"/>
+      <c r="B604" s="8" t="inlineStr"/>
+      <c r="C604" s="8" t="inlineStr">
+        <is>
+          <t>dcfw-xcx-002</t>
+        </is>
+      </c>
+      <c r="D604" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E604" s="8" t="n"/>
+      <c r="F604" s="8" t="inlineStr">
+        <is>
+          <t>验证拒绝位置授权后的引导重新授权流程</t>
+        </is>
+      </c>
+      <c r="G604" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已拒绝位置授权</t>
+        </is>
+      </c>
+      <c r="H604" s="8" t="inlineStr">
+        <is>
+          <t>1. 进入打车页面，检测到无位置权限。
+2. 页面显示"需要位置权限"提示。
+3. 点击"去设置"按钮。
+4. 跳转到微信小程序设置页（wx.openSetting）。
+5. 用户手动开启位置权限。
+6. 返回小程序</t>
+        </is>
+      </c>
+      <c r="I604" s="8" t="inlineStr">
+        <is>
+          <t>1. 页面正确识别无权限状态。
+2. 点击"去设置"打开小程序权限设置页。
+3. 设置页列出"位置信息"开关。
+4. 开启后返回小程序，自动重新获取位置。
+5. 定位成功，页面正常展示</t>
+        </is>
+      </c>
+      <c r="J604" s="8" t="inlineStr">
+        <is>
+          <t>小程序拒绝授权后不能再次弹窗，只能引导去设置</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="8" t="inlineStr"/>
+      <c r="B605" s="8" t="inlineStr"/>
+      <c r="C605" s="8" t="inlineStr">
+        <is>
+          <t>dcfw-xcx-003</t>
+        </is>
+      </c>
+      <c r="D605" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E605" s="8" t="n"/>
+      <c r="F605" s="8" t="inlineStr">
+        <is>
+          <t>验证打车跳转第三方小程序（滴滴/高德）</t>
+        </is>
+      </c>
+      <c r="G605" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已选择目的地
+2. 准备跳转第三方打车</t>
+        </is>
+      </c>
+      <c r="H605" s="8" t="inlineStr">
+        <is>
+          <t>1. 选择"滴滴出行"打车。
+2. 点击"呼叫快车"。
+3. 观察跳转行为</t>
+        </is>
+      </c>
+      <c r="I605" s="8" t="inlineStr">
+        <is>
+          <t>1. 调用wx.navigateToMiniProgram跳转至滴滴小程序。
+2. 微信弹出"即将打开滴滴出行小程序"确认框。
+3. 确认后跳转成功，携带起点/终点参数。
+4. 取消则留在当前小程序。
+5. 从滴滴小程序返回时回到打车页面</t>
+        </is>
+      </c>
+      <c r="J605" s="8" t="inlineStr">
+        <is>
+          <t>跳转其他小程序需用户确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B606" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C606" s="20" t="inlineStr">
+        <is>
+          <t>dypw-xcx-001</t>
+        </is>
+      </c>
+      <c r="D606" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E606" s="20" t="inlineStr">
+        <is>
+          <t>电影票务
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F606" s="20" t="inlineStr">
+        <is>
+          <t>验证电影选座界面在小程序中的触控交互（缩放/拖动）</t>
+        </is>
+      </c>
+      <c r="G606" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户已选择影片和场次
+2. 进入选座页面</t>
+        </is>
+      </c>
+      <c r="H606" s="20" t="inlineStr">
+        <is>
+          <t>1. 查看座位图展示。
+2. 双指捏合缩小座位图。
+3. 双指张开放大座位图。
+4. 单指拖动查看不同区域。
+5. 点击绿色可选座位。
+6. 已选座位高亮标记</t>
+        </is>
+      </c>
+      <c r="I606" s="20" t="inlineStr">
+        <is>
+          <t>1. 座位图在小程序canvas或movable-view中正常渲染。
+2. 双指缩放流畅，无卡顿。
+3. 拖动时不触发页面下拉刷新（需禁止冒泡）。
+4. 点击座位响应准确（不会误触相邻座位）。
+5. 最多选4座，选第5座提示限制。
+6. 已售灰色座位点击无反应</t>
+        </is>
+      </c>
+      <c r="J606" s="20" t="inlineStr">
+        <is>
+          <t>小程序触控事件处理与原生App不同</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="8" t="inlineStr"/>
+      <c r="B607" s="8" t="inlineStr"/>
+      <c r="C607" s="8" t="inlineStr">
+        <is>
+          <t>dypw-xcx-002</t>
+        </is>
+      </c>
+      <c r="D607" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E607" s="8" t="n"/>
+      <c r="F607" s="8" t="inlineStr">
+        <is>
+          <t>验证电影出票后取票码在小程序内展示和保存</t>
+        </is>
+      </c>
+      <c r="G607" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已购票成功
+2. 出票完成</t>
+        </is>
+      </c>
+      <c r="H607" s="8" t="inlineStr">
+        <is>
+          <t>1. 查看订单详情页的取票码/二维码。
+2. 调整手机亮度查看二维码清晰度。
+3. 长按二维码图片。
+4. 点击"保存到手机"（如有该功能）</t>
+        </is>
+      </c>
+      <c r="I607" s="8" t="inlineStr">
+        <is>
+          <t>1. 取票码数字清晰显示，字体大小合适。
+2. 二维码清晰可扫（影院扫码机能识别）。
+3. 小程序可调用wx.setScreenBrightness提高亮度。
+4. 长按二维码弹出保存选项（需相册授权）。
+5. 同时展示短信取票码文本</t>
+        </is>
+      </c>
+      <c r="J607" s="8" t="inlineStr">
+        <is>
+          <t>到影院后需要在小程序内展示取票码给机器扫</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="8" t="inlineStr"/>
+      <c r="B608" s="8" t="inlineStr"/>
+      <c r="C608" s="8" t="inlineStr">
+        <is>
+          <t>dypw-xcx-003</t>
+        </is>
+      </c>
+      <c r="D608" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E608" s="8" t="n"/>
+      <c r="F608" s="8" t="inlineStr">
+        <is>
+          <t>验证选座页面在小程序中实时更新已售座位</t>
+        </is>
+      </c>
+      <c r="G608" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户A和用户B同时浏览同一场次</t>
+        </is>
+      </c>
+      <c r="H608" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户A在选座页面看到某座位可选。
+2. 用户B购买了该座位。
+3. 用户A的页面是否实时更新。
+4. 用户A点击该座位</t>
+        </is>
+      </c>
+      <c r="I608" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户A页面通过WebSocket或轮询检测更新。
+2. 被购买的座位自动变为灰色。
+3. 如用户A选中后提交时座位已被占，提示"该座位已被他人选择，请重新选座"。
+4. 不产生重复出票</t>
+        </is>
+      </c>
+      <c r="J608" s="8" t="inlineStr">
+        <is>
+          <t>小程序可使用wx.connectSocket做实时通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B609" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C609" s="20" t="inlineStr">
+        <is>
+          <t>hycz-xcx-001</t>
+        </is>
+      </c>
+      <c r="D609" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E609" s="20" t="inlineStr">
+        <is>
+          <t>会员充值
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F609" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序内手机号输入键盘和运营商自动识别</t>
+        </is>
+      </c>
+      <c r="G609" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户选择"话费充值"分类
+2. 选择50元面额</t>
+        </is>
+      </c>
+      <c r="H609" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击手机号输入框。
+2. 观察弹出键盘类型。
+3. 输入手机号"13800138000"。
+4. 观察运营商自动识别。
+5. 输入完成后收起键盘</t>
+        </is>
+      </c>
+      <c r="I609" s="20" t="inlineStr">
+        <is>
+          <t>1. 弹出纯数字键盘（type="number"）。
+2. 输入11位后自动收起键盘或限制继续输入。
+3. 输入过程中自动识别运营商："中国移动"。
+4. 运营商标识Icon正确展示。
+5. 键盘收起后页面恢复正常布局</t>
+        </is>
+      </c>
+      <c r="J609" s="20" t="inlineStr">
+        <is>
+          <t>小程序input type="number"不带小数点的纯数字键盘</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="8" t="inlineStr"/>
+      <c r="B610" s="8" t="inlineStr"/>
+      <c r="C610" s="8" t="inlineStr">
+        <is>
+          <t>hycz-xcx-002</t>
+        </is>
+      </c>
+      <c r="D610" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E610" s="8" t="n"/>
+      <c r="F610" s="8" t="inlineStr">
+        <is>
+          <t>验证充值成功后订阅消息通知推送</t>
+        </is>
+      </c>
+      <c r="G610" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已授权订阅消息
+2. 话费充值成功</t>
+        </is>
+      </c>
+      <c r="H610" s="8" t="inlineStr">
+        <is>
+          <t>1. 充值完成后等待通知。
+2. 检查微信"服务通知"。
+3. 点击通知卡片</t>
+        </is>
+      </c>
+      <c r="I610" s="8" t="inlineStr">
+        <is>
+          <t>1. 微信"服务通知"收到充值成功通知（&lt;1分钟）。
+2. 通知内容：充值金额/充值账号/充值状态。
+3. 点击卡片跳转到小程序对应订单详情页。
+4. 详情页展示"充值成功"状态</t>
+        </is>
+      </c>
+      <c r="J610" s="8" t="inlineStr">
+        <is>
+          <t>充值结果通过订阅消息推送给用户</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B611" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C611" s="20" t="inlineStr">
+        <is>
+          <t>jdgw-xcx-001</t>
+        </is>
+      </c>
+      <c r="D611" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E611" s="20" t="inlineStr">
+        <is>
+          <t>家电购物
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F611" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序跳转京东App/京东小程序完成购买</t>
+        </is>
+      </c>
+      <c r="G611" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户在家电购物列表
+2. 手机已安装京东App</t>
+        </is>
+      </c>
+      <c r="H611" s="20" t="inlineStr">
+        <is>
+          <t>1. 点击某家电商品。
+2. 查看商品详情和"预计返利XX元"。
+3. 点击"去购买"。
+4. 观察跳转行为</t>
+        </is>
+      </c>
+      <c r="I611" s="20" t="inlineStr">
+        <is>
+          <t>1. 跳转时携带CPS推广参数（辛贝渠道标识）。
+2. 优先跳转京东App（通过scheme）。
+3. 未安装京东App时跳转京东小程序或H5。
+4. 跳转链接中推广参数正确（用于佣金追踪）。
+5. 返回快乐羊毛小程序时页面恢复</t>
+        </is>
+      </c>
+      <c r="J611" s="20" t="inlineStr">
+        <is>
+          <t>确保CPS推广参数不丢失</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="8" t="inlineStr"/>
+      <c r="B612" s="8" t="inlineStr"/>
+      <c r="C612" s="8" t="inlineStr">
+        <is>
+          <t>jdgw-xcx-002</t>
+        </is>
+      </c>
+      <c r="D612" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E612" s="8" t="n"/>
+      <c r="F612" s="8" t="inlineStr">
+        <is>
+          <t>验证家电商品图片在小程序中的懒加载</t>
+        </is>
+      </c>
+      <c r="G612" s="8" t="inlineStr">
+        <is>
+          <t>1. 家电列表有20+商品，每个有主图</t>
+        </is>
+      </c>
+      <c r="H612" s="8" t="inlineStr">
+        <is>
+          <t>1. 进入家电购物列表。
+2. 观察首屏图片加载。
+3. 快速向下滚动。
+4. 观察屏幕外图片加载行为</t>
+        </is>
+      </c>
+      <c r="I612" s="8" t="inlineStr">
+        <is>
+          <t>1. 首屏内图片优先加载。
+2. 屏幕外图片不立即加载（lazy-load）。
+3. 滚动到视口内时自动加载。
+4. 图片未加载时显示占位图。
+5. 列表滚动流畅不卡顿</t>
+        </is>
+      </c>
+      <c r="J612" s="8" t="inlineStr">
+        <is>
+          <t>小程序image组件支持lazy-load属性</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B613" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C613" s="20" t="inlineStr">
+        <is>
+          <t>gwfl-xcx-001</t>
+        </is>
+      </c>
+      <c r="D613" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E613" s="20" t="inlineStr">
+        <is>
+          <t>购物返利
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F613" s="20" t="inlineStr">
+        <is>
+          <t>验证小程序内粘贴商品链接的剪贴板读取行为</t>
+        </is>
+      </c>
+      <c r="G613" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户已在淘宝/京东App复制了商品链接
+2. 切换到快乐羊毛小程序</t>
+        </is>
+      </c>
+      <c r="H613" s="20" t="inlineStr">
+        <is>
+          <t>1. 切换到快乐羊毛小程序。
+2. 进入购物返利页面。
+3. 点击搜索框/粘贴区域。
+4. 长按粘贴或直接触发自动识别。
+5. 检查链接解析</t>
+        </is>
+      </c>
+      <c r="I613" s="20" t="inlineStr">
+        <is>
+          <t>1. 小程序可通过wx.getClipboardData读取剪贴板。
+2. 微信可能弹出"快乐羊毛要读取你的剪贴板"提示（iOS 14+）。
+3. 用户允许后粘贴内容正确。
+4. 系统解析商品链接，展示商品信息和预计返利。
+5. 生成专属推广链接</t>
+        </is>
+      </c>
+      <c r="J613" s="20" t="inlineStr">
+        <is>
+          <t>iOS 14+有剪贴板读取隐私提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="8" t="inlineStr"/>
+      <c r="B614" s="8" t="inlineStr"/>
+      <c r="C614" s="8" t="inlineStr">
+        <is>
+          <t>gwfl-xcx-002</t>
+        </is>
+      </c>
+      <c r="D614" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E614" s="8" t="n"/>
+      <c r="F614" s="8" t="inlineStr">
+        <is>
+          <t>验证购物返利授权绑定淘宝/京东账号流程</t>
+        </is>
+      </c>
+      <c r="G614" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户首次使用购物返利
+2. 未绑定淘宝/京东账号</t>
+        </is>
+      </c>
+      <c r="H614" s="8" t="inlineStr">
+        <is>
+          <t>1. 进入购物返利功能。
+2. 提示需要绑定平台账号。
+3. 点击"绑定淘宝账号"。
+4. 跳转淘宝授权页面（web-view）。
+5. 完成授权后返回小程序</t>
+        </is>
+      </c>
+      <c r="I614" s="8" t="inlineStr">
+        <is>
+          <t>1. 绑定提示清晰告知用途。
+2. 通过web-view打开淘宝联盟授权页。
+3. 用户在web-view中完成淘宝登录授权。
+4. 授权回调返回小程序，绑定成功。
+5. 显示已绑定状态</t>
+        </is>
+      </c>
+      <c r="J614" s="8" t="inlineStr">
+        <is>
+          <t>第三方授权在小程序中通过web-view实现</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B615" s="20" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="C615" s="20" t="inlineStr">
+        <is>
+          <t>grzx-xcx-001</t>
+        </is>
+      </c>
+      <c r="D615" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E615" s="20" t="inlineStr">
+        <is>
+          <t>个人中心
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F615" s="20" t="inlineStr">
+        <is>
+          <t>验证微信一键登录获取手机号的完整流程</t>
+        </is>
+      </c>
+      <c r="G615" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户首次打开小程序
+2. 未注册过</t>
+        </is>
+      </c>
+      <c r="H615" s="20" t="inlineStr">
+        <is>
+          <t>1. 进入小程序，显示登录页。
+2. 点击"微信一键登录"按钮（button open-type="getPhoneNumber"）。
+3. 微信弹出手机号授权弹窗。
+4. 点击"允许"。
+5. 登录成功跳转首页</t>
+        </is>
+      </c>
+      <c r="I615" s="20" t="inlineStr">
+        <is>
+          <t>1. 登录按钮使用小程序原生&lt;button&gt;组件。
+2. 微信弹出"快乐羊毛申请获取你的手机号"授权框。
+3. 允许后获取加密手机号数据（encryptedData+iv）。
+4. 后端解密得到手机号，自动注册新用户。
+5. 登录成功，个人中心显示脱敏手机号（138****8000）</t>
+        </is>
+      </c>
+      <c r="J615" s="20" t="inlineStr">
+        <is>
+          <t>小程序获取手机号必须用&lt;button&gt;组件，不能js直接调用</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="8" t="inlineStr"/>
+      <c r="B616" s="8" t="inlineStr"/>
+      <c r="C616" s="8" t="inlineStr">
+        <is>
+          <t>grzx-xcx-002</t>
+        </is>
+      </c>
+      <c r="D616" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E616" s="8" t="n"/>
+      <c r="F616" s="8" t="inlineStr">
+        <is>
+          <t>验证推广海报生成并保存到相册（wx.saveImageToPhotosAlbum）</t>
+        </is>
+      </c>
+      <c r="G616" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户已登录
+2. 进入推广中心页面</t>
+        </is>
+      </c>
+      <c r="H616" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击"生成推广海报"。
+2. 等待海报生成（canvas绘制）。
+3. 海报展示个人专属二维码。
+4. 点击"保存到相册"。
+5. 首次弹出相册写入授权</t>
+        </is>
+      </c>
+      <c r="I616" s="8" t="inlineStr">
+        <is>
+          <t>1. 海报通过canvas绘制完成。
+2. 海报包含个人专属二维码（唯一、可识别）。
+3. 点击保存弹出微信授权"保存到相册"。
+4. 允许后保存成功，提示"已保存到相册"。
+5. 拒绝授权时提示"请在设置中开启相册权限"</t>
+        </is>
+      </c>
+      <c r="J616" s="8" t="inlineStr">
+        <is>
+          <t>小程序saveImage需要scope.writePhotosAlbum授权</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="8" t="inlineStr"/>
+      <c r="B617" s="8" t="inlineStr"/>
+      <c r="C617" s="8" t="inlineStr">
+        <is>
+          <t>grzx-xcx-003</t>
+        </is>
+      </c>
+      <c r="D617" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E617" s="8" t="n"/>
+      <c r="F617" s="8" t="inlineStr">
+        <is>
+          <t>验证订单列表下拉刷新和分页加载交互</t>
+        </is>
+      </c>
+      <c r="G617" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户有10+笔订单
+2. 在"我的订单"页面</t>
+        </is>
+      </c>
+      <c r="H617" s="8" t="inlineStr">
+        <is>
+          <t>1. 下拉刷新订单列表。
+2. 观察刷新动画。
+3. 滚动到底部加载更多。
+4. 按状态Tab切换筛选。
+5. 按订单类型筛选</t>
+        </is>
+      </c>
+      <c r="I617" s="8" t="inlineStr">
+        <is>
+          <t>1. 下拉显示微信原生刷新动画。
+2. 刷新后列表更新为最新数据。
+3. 触底自动加载下一页。
+4. 切换状态Tab筛选正确（待支付/已完成/已退款等）。
+5. 按业务线筛选正确（外卖券/充值/餐饮等）</t>
+        </is>
+      </c>
+      <c r="J617" s="8" t="inlineStr">
+        <is>
+          <t>订单列表是高频访问页面</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="8" t="inlineStr"/>
+      <c r="B618" s="8" t="inlineStr"/>
+      <c r="C618" s="8" t="inlineStr">
+        <is>
+          <t>grzx-xcx-004</t>
+        </is>
+      </c>
+      <c r="D618" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E618" s="8" t="n"/>
+      <c r="F618" s="8" t="inlineStr">
+        <is>
+          <t>验证小程序分享推广海报/推广链接到微信好友</t>
+        </is>
+      </c>
+      <c r="G618" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户在推广中心
+2. 已生成推广二维码</t>
+        </is>
+      </c>
+      <c r="H618" s="8" t="inlineStr">
+        <is>
+          <t>1. 点击"分享给好友"按钮。
+2. 选择好友发送分享卡片。
+3. 好友点击卡片进入小程序。
+4. 好友注册后检查推广关系</t>
+        </is>
+      </c>
+      <c r="I618" s="8" t="inlineStr">
+        <is>
+          <t>1. 分享卡片标题和描述正确（如"快来快乐羊毛省钱"）。
+2. 卡片携带推广者ID参数。
+3. 好友点击后进入小程序并绑定推广关系。
+4. 推广中心"我的团队"新增该好友。
+5. 好友消费后推广者可获得佣金</t>
+        </is>
+      </c>
+      <c r="J618" s="8" t="inlineStr">
+        <is>
+          <t>分享裂变是获客核心——参数传递不能丢</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="8" t="inlineStr"/>
+      <c r="B619" s="8" t="inlineStr"/>
+      <c r="C619" s="8" t="inlineStr">
+        <is>
+          <t>grzx-xcx-005</t>
+        </is>
+      </c>
+      <c r="D619" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E619" s="8" t="n"/>
+      <c r="F619" s="8" t="inlineStr">
+        <is>
+          <t>验证佣金/余额数据在小程序端实时更新</t>
+        </is>
+      </c>
+      <c r="G619" s="8" t="inlineStr">
+        <is>
+          <t>1. 用户是代理商
+2. 有佣金记录</t>
+        </is>
+      </c>
+      <c r="H619" s="8" t="inlineStr">
+        <is>
+          <t>1. 查看个人中心"预估收入"和"可提现余额"。
+2. 通过另一个账号完成一笔新订单。
+3. 下拉刷新个人中心。
+4. 检查佣金变化</t>
+        </is>
+      </c>
+      <c r="I619" s="8" t="inlineStr">
+        <is>
+          <t>1. "预估收入"和"可提现余额"正确展示。
+2. 新订单完成后下拉刷新。
+3. "预估收入"增加相应佣金金额。
+4. 数据与后台管理端完全一致。
+5. 金额精确到分（0.00格式）</t>
+        </is>
+      </c>
+      <c r="J619" s="8" t="inlineStr">
+        <is>
+          <t>佣金准确性直接影响用户信任</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="20" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B620" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C620" s="20" t="inlineStr">
+        <is>
+          <t>jycz-xcx-001</t>
+        </is>
+      </c>
+      <c r="D620" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E620" s="20" t="inlineStr">
+        <is>
+          <t>加油/充电
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F620" s="20" t="inlineStr">
+        <is>
+          <t>验证加油站/充电桩列表的位置排序（wx.getLocation）</t>
+        </is>
+      </c>
+      <c r="G620" s="20" t="inlineStr">
+        <is>
+          <t>1. 用户已授权位置权限
+2. 附近有加油站/充电桩数据</t>
+        </is>
+      </c>
+      <c r="H620" s="20" t="inlineStr">
+        <is>
+          <t>1. 进入加油/充电页面。
+2. 系统获取当前位置。
+3. 展示附近站点列表。
+4. 检查排序是否按距离</t>
+        </is>
+      </c>
+      <c r="I620" s="20" t="inlineStr">
+        <is>
+          <t>1. 位置获取成功。
+2. 列表按距离从近到远排序。
+3. 每项展示名称+距离（如"中石化加油站 1.2km"）。
+4. 点击某站点跳转第三方App/H5（携带CPS参数）</t>
+        </is>
+      </c>
+      <c r="J620" s="20" t="inlineStr">
+        <is>
+          <t>复用打车模块的位置授权</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="20" t="inlineStr">
+        <is>
+          <t>商家端</t>
+        </is>
+      </c>
+      <c r="B621" s="20" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="C621" s="20" t="inlineStr">
+        <is>
+          <t>sjd-xcx-001</t>
+        </is>
+      </c>
+      <c r="D621" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E621" s="20" t="inlineStr">
+        <is>
+          <t>商家端收银台
+(小程序环境)</t>
+        </is>
+      </c>
+      <c r="F621" s="20" t="inlineStr">
+        <is>
+          <t>验证商家端小程序收银台生成二维码的完整交互</t>
+        </is>
+      </c>
+      <c r="G621" s="20" t="inlineStr">
+        <is>
+          <t>1. 商家品牌主账号/门店子账号已登录商家端小程序</t>
+        </is>
+      </c>
+      <c r="H621" s="20" t="inlineStr">
+        <is>
+          <t>1. 进入收银台页面。
+2. 点击金额输入框，弹出数字键盘。
+3. 输入消费金额100。
+4. 系统自动展示折扣计算（8折=实付80元）。
+5. 点击"生成收款码"按钮。
+6. 等待二维码生成。
+7. 展示二维码和15分钟倒计时</t>
+        </is>
+      </c>
+      <c r="I621" s="20" t="inlineStr">
+        <is>
+          <t>1. 数字键盘正常弹出（带小数点）。
+2. 输入金额后折扣实时计算并展示。
+3. 点击生成后按钮变为loading状态。
+4. 二维码生成成功，清晰可扫。
+5. 倒计时正确显示"14:59"并倒数。
+6. 页面布局适配不同手机屏幕</t>
+        </is>
+      </c>
+      <c r="J621" s="20" t="inlineStr">
+        <is>
+          <t>收银台是商家最高频使用的功能</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="8" t="inlineStr"/>
+      <c r="B622" s="8" t="inlineStr"/>
+      <c r="C622" s="8" t="inlineStr">
+        <is>
+          <t>sjd-xcx-002</t>
+        </is>
+      </c>
+      <c r="D622" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E622" s="8" t="n"/>
+      <c r="F622" s="8" t="inlineStr">
+        <is>
+          <t>验证商家端小程序验证码核销输入交互</t>
+        </is>
+      </c>
+      <c r="G622" s="8" t="inlineStr">
+        <is>
+          <t>1. 有一笔人工辅助订单已下发验证码
+2. 用户到店出示验证码</t>
+        </is>
+      </c>
+      <c r="H622" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家在订单管理中找到该订单。
+2. 点击"核销"按钮。
+3. 输入用户出示的验证码。
+4. 点击"确认核销"。
+5. 等待结果</t>
+        </is>
+      </c>
+      <c r="I622" s="8" t="inlineStr">
+        <is>
+          <t>1. 弹出验证码输入框，自动获取焦点。
+2. 数字键盘弹出。
+3. 输入完成后"确认核销"按钮可点击。
+4. 点击后按钮loading防重复。
+5. 核销成功弹出Toast"核销成功"。
+6. 订单状态自动刷新为"已完成"</t>
+        </is>
+      </c>
+      <c r="J622" s="8" t="inlineStr">
+        <is>
+          <t>核销操作需要快速简洁</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="8" t="inlineStr"/>
+      <c r="B623" s="8" t="inlineStr"/>
+      <c r="C623" s="8" t="inlineStr">
+        <is>
+          <t>sjd-xcx-003</t>
+        </is>
+      </c>
+      <c r="D623" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E623" s="8" t="n"/>
+      <c r="F623" s="8" t="inlineStr">
+        <is>
+          <t>验证商家端小程序订单管理列表的筛选交互</t>
+        </is>
+      </c>
+      <c r="G623" s="8" t="inlineStr">
+        <is>
+          <t>1. 商家端小程序已登录
+2. 有多笔订单</t>
+        </is>
+      </c>
+      <c r="H623" s="8" t="inlineStr">
+        <is>
+          <t>1. 进入订单管理页面。
+2. 点击日期筛选，选择日期范围。
+3. 点击状态筛选（已支付/已退款等）。
+4. 下拉刷新列表。
+5. 滚动到底部加载更多</t>
+        </is>
+      </c>
+      <c r="I623" s="8" t="inlineStr">
+        <is>
+          <t>1. 日期选择器使用小程序picker组件（mode="date"）。
+2. 状态筛选正常工作。
+3. 下拉刷新显示微信原生动画。
+4. 触底加载分页数据。
+5. 只显示本门店数据</t>
+        </is>
+      </c>
+      <c r="J623" s="8" t="inlineStr">
+        <is>
+          <t>小程序picker的日期选择器交互</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="8" t="inlineStr"/>
+      <c r="B624" s="8" t="inlineStr"/>
+      <c r="C624" s="8" t="inlineStr">
+        <is>
+          <t>sjd-xcx-004</t>
+        </is>
+      </c>
+      <c r="D624" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E624" s="8" t="n"/>
+      <c r="F624" s="8" t="inlineStr">
+        <is>
+          <t>验证门店子账号登录商家端小程序的权限隔离</t>
+        </is>
+      </c>
+      <c r="G624" s="8" t="inlineStr">
+        <is>
+          <t>1. 品牌有门店A和门店B
+2. 使用门店A的子账号登录</t>
+        </is>
+      </c>
+      <c r="H624" s="8" t="inlineStr">
+        <is>
+          <t>1. 门店A子账号登录商家端小程序。
+2. 查看订单管理——只显示门店A订单。
+3. 查看数据统计——只显示门店A流水。
+4. 检查菜单——无"创建子账号"功能。
+5. 检查收银台——无"修正金额"按钮</t>
+        </is>
+      </c>
+      <c r="I624" s="8" t="inlineStr">
+        <is>
+          <t>1. 订单列表只展示门店A的数据。
+2. 数据统计只有门店A的流水和核销笔数。
+3. 菜单中无子账号管理入口。
+4. 收银台无手动修正金额功能。
+5. 通过修改API参数尝试查看门店B数据返回"无权限"</t>
+        </is>
+      </c>
+      <c r="J624" s="8" t="inlineStr">
+        <is>
+          <t>数据隔离在小程序端也必须严格执行</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="20" t="inlineStr">
+        <is>
+          <t>管理后台</t>
+        </is>
+      </c>
+      <c r="B625" s="20" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C625" s="20" t="inlineStr">
+        <is>
+          <t>htgl-pc-001</t>
+        </is>
+      </c>
+      <c r="D625" s="20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E625" s="20" t="inlineStr">
+        <is>
+          <t>管理后台
+(PC浏览器环境)</t>
+        </is>
+      </c>
+      <c r="F625" s="20" t="inlineStr">
+        <is>
+          <t>验证管理后台登录和核心操作在Chrome浏览器正常运行</t>
+        </is>
+      </c>
+      <c r="G625" s="20" t="inlineStr">
+        <is>
+          <t>1. Chrome最新版浏览器
+2. 访问 https://red.jinyedaojia.com/</t>
+        </is>
+      </c>
+      <c r="H625" s="20" t="inlineStr">
+        <is>
+          <t>1. 输入admin/admin123登录。
+2. 查看订单列表并翻页。
+3. 执行分佣配置修改。
+4. 查看选品仓库。
+5. 查看退款审核列表</t>
+        </is>
+      </c>
+      <c r="I625" s="20" t="inlineStr">
+        <is>
+          <t>1. 登录成功进入后台首页。
+2. 订单列表分页正常（首屏加载&lt;3秒）。
+3. 分佣配置保存成功。
+4. 选品仓库列表正常。
+5. 退款列表可正常审核操作。
+6. 页面布局完整无错位</t>
+        </is>
+      </c>
+      <c r="J625" s="20" t="inlineStr">
+        <is>
+          <t>后台测试环境: https://red.jinyedaojia.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="8" t="inlineStr"/>
+      <c r="B626" s="8" t="inlineStr"/>
+      <c r="C626" s="8" t="inlineStr">
+        <is>
+          <t>htgl-pc-002</t>
+        </is>
+      </c>
+      <c r="D626" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E626" s="8" t="n"/>
+      <c r="F626" s="8" t="inlineStr">
+        <is>
+          <t>验证管理后台Excel文件上传/下载功能在浏览器中正常</t>
+        </is>
+      </c>
+      <c r="G626" s="8" t="inlineStr">
+        <is>
+          <t>1. Chrome浏览器已登录后台
+2. 准备测试Excel文件</t>
+        </is>
+      </c>
+      <c r="H626" s="8" t="inlineStr">
+        <is>
+          <t>1. 在佣金导入页面点击"选择文件"。
+2. 浏览器弹出文件选择框。
+3. 选择Excel文件上传。
+4. 在对账管理页面点击"导出"。
+5. 检查浏览器下载</t>
+        </is>
+      </c>
+      <c r="I626" s="8" t="inlineStr">
+        <is>
+          <t>1. 文件选择框正常弹出。
+2. 选择.xlsx文件后正常上传解析。
+3. 导出Excel正常下载到本地。
+4. 下载文件名含日期标识。
+5. 打开Excel数据完整，中文无乱码</t>
+        </is>
+      </c>
+      <c r="J626" s="8" t="inlineStr">
+        <is>
+          <t>上传/下载是后台常见操作</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="8" t="inlineStr"/>
+      <c r="B627" s="8" t="inlineStr"/>
+      <c r="C627" s="8" t="inlineStr">
+        <is>
+          <t>htgl-pc-003</t>
+        </is>
+      </c>
+      <c r="D627" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E627" s="8" t="n"/>
+      <c r="F627" s="8" t="inlineStr">
+        <is>
+          <t>验证管理后台在Edge浏览器的兼容性</t>
+        </is>
+      </c>
+      <c r="G627" s="8" t="inlineStr">
+        <is>
+          <t>1. Edge最新版浏览器
+2. 管理员账号</t>
+        </is>
+      </c>
+      <c r="H627" s="8" t="inlineStr">
+        <is>
+          <t>1. 在Edge中访问后台登录。
+2. 查看订单列表和数据报表。
+3. 执行退款审核操作。
+4. 查看选品仓库并执行一键同步。
+5. 上传Excel文件</t>
+        </is>
+      </c>
+      <c r="I627" s="8" t="inlineStr">
+        <is>
+          <t>1. 所有页面布局与Chrome一致。
+2. 表格渲染正常。
+3. 退款审核弹窗正常显示。
+4. 同步进度条正常。
+5. 文件上传正常</t>
+        </is>
+      </c>
+      <c r="J627" s="8" t="inlineStr">
+        <is>
+          <t>确保Chrome和Edge两个主流浏览器都兼容</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J453"/>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="E67:E90"/>
     <mergeCell ref="A552:J552"/>
     <mergeCell ref="E20:E37"/>
     <mergeCell ref="E38:E56"/>
+    <mergeCell ref="A582:J582"/>
     <mergeCell ref="A455:J455"/>
     <mergeCell ref="E2:E19"/>
     <mergeCell ref="E57:E65"/>
@@ -26180,7 +28570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="29.125" customWidth="1" style="3" min="2" max="4"/>
@@ -27123,6 +29513,248 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="B59" s="10">
+        <f>== 各模块·小程序环境专项用例 ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>免费资料区(小程序环境): 下拉刷新/页面栈/剪贴板/分享</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>外卖红包(小程序环境): App跳转/scheme/降级H5/分享卡片</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>通用券(小程序环境): 微信支付交互/取消重付/剪贴板/协议勾选</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>餐饮直连(小程序环境): 扫码/微信扫一扫/前后台切换/数字键盘</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>餐饮人工辅助(小程序环境): chooseImage/预览/订阅消息/降级/核销</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>打车服务(小程序环境): 位置授权/openSetting/跳转其他小程序</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>电影票务(小程序环境): 触控选座/取票码展示/实时座位</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>会员充值(小程序环境): 数字键盘/运营商识别/订阅消息</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>家电购物(小程序环境): 跳转京东/懒加载</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>购物返利(小程序环境): 剪贴板读取/web-view授权</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>个人中心(小程序环境): 手机号授权/海报canvas/保存相册/分享裂变</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>加油充电(小程序环境): 位置排序</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>商家端</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>商家端收银台(小程序环境): 二维码生成/核销输入/订单筛选/权限隔离</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>管理后台</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>管理后台(PC浏览器): Chrome/Edge兼容/上传下载</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>各模块小程序环境小计</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>★ 完善版v2 最终总计 ★</t>
+        </is>
+      </c>
+      <c r="C76" s="15">
+        <f>574+45-2</f>
+        <v/>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>原574 - 去重2 + 模块小程序环境45</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto commit: 2026-03-20 10:15:55
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -225,8 +225,14 @@
       <color rgb="000D47A1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00E65100"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="38">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -447,6 +453,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00BBDEFB"/>
         <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E65100"/>
+        <bgColor rgb="00E65100"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -777,7 +795,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -826,6 +844,13 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1276,7 +1301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J571"/>
+  <dimension ref="A1:J593"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="6.5" customWidth="1" style="3" min="1" max="3"/>
@@ -20170,50 +20195,15 @@
     </row>
     <row r="455">
       <c r="A455" s="8" t="inlineStr"/>
-      <c r="B455" s="8" t="inlineStr"/>
-      <c r="C455" s="8" t="inlineStr">
-        <is>
-          <t>wlyc-005</t>
-        </is>
-      </c>
-      <c r="D455" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E455" s="8" t="n"/>
-      <c r="F455" s="8" t="inlineStr">
-        <is>
-          <t>验证断网环境下凭证图片上传的处理</t>
-        </is>
-      </c>
-      <c r="G455" s="8" t="inlineStr">
-        <is>
-          <t>1. 用户在人工辅助模式下单页
-2. 已输入消费金额</t>
-        </is>
-      </c>
-      <c r="H455" s="8" t="inlineStr">
-        <is>
-          <t>1. 选择一张凭证图片开始上传。
-2. 上传过程中断开网络。
-3. 观察上传结果提示。
-4. 恢复网络后重新上传</t>
-        </is>
-      </c>
-      <c r="I455" s="8" t="inlineStr">
-        <is>
-          <t>1. 上传失败，提示"网络异常，上传失败"。
-2. 已上传成功的图片不受影响（如有多张）。
-3. 恢复网络后可重新选择上传。
-4. 不产生损坏的图片数据</t>
-        </is>
-      </c>
-      <c r="J455" s="8" t="inlineStr">
-        <is>
-          <t>验证图片上传的断点续传或失败回滚</t>
-        </is>
-      </c>
+      <c r="B455" s="16" t="n"/>
+      <c r="C455" s="16" t="n"/>
+      <c r="D455" s="16" t="n"/>
+      <c r="E455" s="16" t="n"/>
+      <c r="F455" s="16" t="n"/>
+      <c r="G455" s="16" t="n"/>
+      <c r="H455" s="16" t="n"/>
+      <c r="I455" s="16" t="n"/>
+      <c r="J455" s="17" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="8" t="inlineStr"/>
@@ -23717,7 +23707,6 @@
         </is>
       </c>
     </row>
-    <row r="526"/>
     <row r="527">
       <c r="A527" s="9" t="inlineStr">
         <is>
@@ -23734,7 +23723,6 @@
       <c r="I527" s="16" t="n"/>
       <c r="J527" s="17" t="n"/>
     </row>
-    <row r="528"/>
     <row r="529">
       <c r="A529" s="18" t="inlineStr">
         <is>
@@ -24891,51 +24879,15 @@
     </row>
     <row r="552">
       <c r="A552" s="8" t="inlineStr"/>
-      <c r="B552" s="8" t="inlineStr"/>
-      <c r="C552" s="8" t="inlineStr">
-        <is>
-          <t>dypw-xcx-002</t>
-        </is>
-      </c>
-      <c r="D552" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E552" s="8" t="n"/>
-      <c r="F552" s="8" t="inlineStr">
-        <is>
-          <t>验证电影出票后取票码在小程序内展示和保存</t>
-        </is>
-      </c>
-      <c r="G552" s="8" t="inlineStr">
-        <is>
-          <t>1. 用户已购票成功
-2. 出票完成</t>
-        </is>
-      </c>
-      <c r="H552" s="8" t="inlineStr">
-        <is>
-          <t>1. 查看订单详情页的取票码/二维码。
-2. 调整手机亮度查看二维码清晰度。
-3. 长按二维码图片。
-4. 点击"保存到手机"（如有该功能）</t>
-        </is>
-      </c>
-      <c r="I552" s="8" t="inlineStr">
-        <is>
-          <t>1. 取票码数字清晰显示，字体大小合适。
-2. 二维码清晰可扫（影院扫码机能识别）。
-3. 小程序可调用wx.setScreenBrightness提高亮度。
-4. 长按二维码弹出保存选项（需相册授权）。
-5. 同时展示短信取票码文本</t>
-        </is>
-      </c>
-      <c r="J552" s="8" t="inlineStr">
-        <is>
-          <t>到影院后需要在小程序内展示取票码给机器扫</t>
-        </is>
-      </c>
+      <c r="B552" s="16" t="n"/>
+      <c r="C552" s="16" t="n"/>
+      <c r="D552" s="16" t="n"/>
+      <c r="E552" s="16" t="n"/>
+      <c r="F552" s="16" t="n"/>
+      <c r="G552" s="16" t="n"/>
+      <c r="H552" s="16" t="n"/>
+      <c r="I552" s="16" t="n"/>
+      <c r="J552" s="17" t="n"/>
     </row>
     <row r="553">
       <c r="A553" s="8" t="inlineStr"/>
@@ -25952,11 +25904,519 @@
         </is>
       </c>
     </row>
+    <row r="582"/>
+    <row r="584">
+      <c r="A584" s="23" t="inlineStr">
+        <is>
+          <t>═══ 复盘补漏 · 需求文档/测试策略交叉比对发现的遗漏点 ═══</t>
+        </is>
+      </c>
+      <c r="B584" s="24" t="n"/>
+      <c r="C584" s="24" t="n"/>
+      <c r="D584" s="24" t="n"/>
+      <c r="E584" s="24" t="n"/>
+      <c r="F584" s="24" t="n"/>
+      <c r="G584" s="24" t="n"/>
+      <c r="H584" s="24" t="n"/>
+      <c r="I584" s="24" t="n"/>
+      <c r="J584" s="24" t="n"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="25" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B585" s="25" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C585" s="25" t="inlineStr">
+        <is>
+          <t>mfzl-bl-001</t>
+        </is>
+      </c>
+      <c r="D585" s="25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E585" s="25" t="inlineStr">
+        <is>
+          <t>免费资料区
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F585" s="25" t="inlineStr">
+        <is>
+          <t>验证快速切换分类Tab时数据请求无竞态条件</t>
+        </is>
+      </c>
+      <c r="G585" s="25" t="inlineStr">
+        <is>
+          <t>1. 免费资料区已配置3个分类
+2. 每个分类各有数据</t>
+        </is>
+      </c>
+      <c r="H585" s="25" t="inlineStr">
+        <is>
+          <t>1. 快速连续点击"学习资料"→"工具模板"→"行业报告"→"全部"，每次间隔&lt;0.5秒。
+2. 最终停留在"全部"分类。
+3. 检查列表数据</t>
+        </is>
+      </c>
+      <c r="I585" s="25" t="inlineStr">
+        <is>
+          <t>1. 列表最终显示"全部"分类数据。
+2. 不出现"工具模板"分类的数据残留在"全部"列表中。
+3. 不出现数据闪烁或重叠。
+4. 无JS报错</t>
+        </is>
+      </c>
+      <c r="J585" s="25" t="inlineStr">
+        <is>
+          <t>需求2.1.4测试关注点：快速切换Tab竞态条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="25" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B586" s="25" t="inlineStr"/>
+      <c r="C586" s="25" t="inlineStr">
+        <is>
+          <t>wamtyj-bl-001</t>
+        </is>
+      </c>
+      <c r="D586" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E586" s="25" t="inlineStr">
+        <is>
+          <t>外卖区-通用券
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F586" s="25" t="inlineStr">
+        <is>
+          <t>验证订单详情页"再次购买"按钮功能</t>
+        </is>
+      </c>
+      <c r="G586" s="25" t="inlineStr">
+        <is>
+          <t>1. 用户已购买过10元通用券
+2. 进入该订单详情页</t>
+        </is>
+      </c>
+      <c r="H586" s="25" t="inlineStr">
+        <is>
+          <t>1. 查看订单详情页。
+2. 点击"再次购买"按钮。
+3. 检查跳转页面</t>
+        </is>
+      </c>
+      <c r="I586" s="25" t="inlineStr">
+        <is>
+          <t>1. "再次购买"按钮可见。
+2. 点击后跳转到该商品的购买页面。
+3. 面额默认选中上次购买的面额（10元）。
+4. 可正常发起新的购买</t>
+        </is>
+      </c>
+      <c r="J586" s="25" t="inlineStr">
+        <is>
+          <t>需求2.2.2：订单详情页操作按钮包含再次购买</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="25" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B587" s="25" t="inlineStr"/>
+      <c r="C587" s="25" t="inlineStr">
+        <is>
+          <t>cyzkrg-bl-001</t>
+        </is>
+      </c>
+      <c r="D587" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E587" s="25" t="inlineStr">
+        <is>
+          <t>餐饮折扣-人工辅助
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F587" s="25" t="inlineStr">
+        <is>
+          <t>验证同名商家是否允许重复录入</t>
+        </is>
+      </c>
+      <c r="G587" s="25" t="inlineStr">
+        <is>
+          <t>1. 已录入一个商家"张三烤肉店"</t>
+        </is>
+      </c>
+      <c r="H587" s="25" t="inlineStr">
+        <is>
+          <t>1. 再次录入一个同名商家"张三烤肉店"（不同地址）。
+2. 提交审核。
+3. 检查结果</t>
+        </is>
+      </c>
+      <c r="I587" s="25" t="inlineStr">
+        <is>
+          <t>1. 允许录入（不同门店可能同名）并提交成功。
+2. 或系统提示"已存在同名商家，是否继续？"。
+3. 列表中两个同名商家可通过地址区分</t>
+        </is>
+      </c>
+      <c r="J587" s="25" t="inlineStr">
+        <is>
+          <t>需求2.3.3测试关注点：同名商家重复录入</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="25" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B588" s="25" t="inlineStr"/>
+      <c r="C588" s="25" t="inlineStr">
+        <is>
+          <t>dcfw-bl-001</t>
+        </is>
+      </c>
+      <c r="D588" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E588" s="25" t="inlineStr">
+        <is>
+          <t>打车服务
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F588" s="25" t="inlineStr">
+        <is>
+          <t>验证定位不精确时支持手动修改起点地址</t>
+        </is>
+      </c>
+      <c r="G588" s="25" t="inlineStr">
+        <is>
+          <t>1. 用户已授权位置并完成定位
+2. 定位结果与实际位置有偏差</t>
+        </is>
+      </c>
+      <c r="H588" s="25" t="inlineStr">
+        <is>
+          <t>1. 查看当前定位地址。
+2. 点击起点地址栏进行修改。
+3. 输入正确地址或在地图上重新选点。
+4. 确认新起点</t>
+        </is>
+      </c>
+      <c r="I588" s="25" t="inlineStr">
+        <is>
+          <t>1. 起点地址栏可点击编辑。
+2. 支持输入文字搜索地址（联想补全）。
+3. 修改后起点更新为新地址。
+4. 跳转第三方打车时使用修改后的地址</t>
+        </is>
+      </c>
+      <c r="J588" s="25" t="inlineStr">
+        <is>
+          <t>需求2.4：定位不精确支持手动修改起点</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="25" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B589" s="25" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="C589" s="25" t="inlineStr">
+        <is>
+          <t>dypw-bl-001</t>
+        </is>
+      </c>
+      <c r="D589" s="25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E589" s="25" t="inlineStr">
+        <is>
+          <t>电影票务
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F589" s="25" t="inlineStr">
+        <is>
+          <t>验证选座最多4座限制及取消已选座位</t>
+        </is>
+      </c>
+      <c r="G589" s="25" t="inlineStr">
+        <is>
+          <t>1. 用户在选座页面
+2. 有多个可选座位</t>
+        </is>
+      </c>
+      <c r="H589" s="25" t="inlineStr">
+        <is>
+          <t>1. 依次选择4个座位，每选一个观察已选列表。
+2. 尝试选第5个座位。
+3. 取消其中1个已选座位。
+4. 再选一个新座位</t>
+        </is>
+      </c>
+      <c r="I589" s="25" t="inlineStr">
+        <is>
+          <t>1. 选择4座后已选列表显示4个座位号。
+2. 选第5个时提示"最多可选4个座位"。
+3. 点击已选座位可取消（高亮恢复为绿色可选）。
+4. 取消后可重新选择新座位</t>
+        </is>
+      </c>
+      <c r="J589" s="25" t="inlineStr">
+        <is>
+          <t>需求2.5：最多4座限制+取消已选座位交互</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="8" t="inlineStr">
+        <is>
+          <t>用户端</t>
+        </is>
+      </c>
+      <c r="B590" s="8" t="inlineStr"/>
+      <c r="C590" s="8" t="inlineStr">
+        <is>
+          <t>dypw-bl-002</t>
+        </is>
+      </c>
+      <c r="D590" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E590" s="8" t="n"/>
+      <c r="F590" s="8" t="inlineStr">
+        <is>
+          <t>验证已过开场时间的场次不可购买</t>
+        </is>
+      </c>
+      <c r="G590" s="8" t="inlineStr">
+        <is>
+          <t>1. 某影片有一个已过开场时间的场次（如开场时间14:00，当前15:00）</t>
+        </is>
+      </c>
+      <c r="H590" s="8" t="inlineStr">
+        <is>
+          <t>1. 查看该影片的场次列表。
+2. 观察已过开场时间的场次展示。
+3. 尝试点击该场次</t>
+        </is>
+      </c>
+      <c r="I590" s="8" t="inlineStr">
+        <is>
+          <t>1. 已过场次显示为灰色/置灰状态。
+2. 标注"已过期"或"已开场"。
+3. 点击后无法进入选座页面，或提示"该场次已开场"</t>
+        </is>
+      </c>
+      <c r="J590" s="8" t="inlineStr">
+        <is>
+          <t>需求2.5测试关注点：场次已过开场时间的处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="25" t="inlineStr">
+        <is>
+          <t>商家端</t>
+        </is>
+      </c>
+      <c r="B591" s="25" t="inlineStr"/>
+      <c r="C591" s="25" t="inlineStr">
+        <is>
+          <t>sjmd-bl-001</t>
+        </is>
+      </c>
+      <c r="D591" s="25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E591" s="25" t="inlineStr">
+        <is>
+          <t>商家端-数据统计
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F591" s="25" t="inlineStr">
+        <is>
+          <t>验证今日流水/本月流水统计的时间起止点（0:00-23:59）</t>
+        </is>
+      </c>
+      <c r="G591" s="25" t="inlineStr">
+        <is>
+          <t>1. 商家端已登录
+2. 有跨日期的订单数据（如23:58下单和00:02下单）</t>
+        </is>
+      </c>
+      <c r="H591" s="25" t="inlineStr">
+        <is>
+          <t>1. 查看"今日流水"数据。
+2. 确认23:58的订单是否计入今日。
+3. 确认00:02的订单是否计入今日（次日查看时）。
+4. 查看"本月流水"，确认月初和月末边界</t>
+        </is>
+      </c>
+      <c r="I591" s="25" t="inlineStr">
+        <is>
+          <t>1. 今日统计范围：当日00:00:00至23:59:59。
+2. 23:58的订单计入当日。
+3. 00:02的订单计入次日。
+4. 本月统计：当月1日00:00至当月最后一日23:59:59</t>
+        </is>
+      </c>
+      <c r="J591" s="25" t="inlineStr">
+        <is>
+          <t>需求3.4测试关注点：统计时间起止点</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="25" t="inlineStr">
+        <is>
+          <t>管理后台</t>
+        </is>
+      </c>
+      <c r="B592" s="25" t="inlineStr"/>
+      <c r="C592" s="25" t="inlineStr">
+        <is>
+          <t>fyxt-bl-001</t>
+        </is>
+      </c>
+      <c r="D592" s="25" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E592" s="25" t="inlineStr">
+        <is>
+          <t>分佣系统
+(复盘补漏)</t>
+        </is>
+      </c>
+      <c r="F592" s="25" t="inlineStr">
+        <is>
+          <t>验证利润为0（实付=成本）时所有角色佣金均为0</t>
+        </is>
+      </c>
+      <c r="G592" s="25" t="inlineStr">
+        <is>
+          <t>1. 后台已配置平台50%/代理商50%
+2. 有一级分销员10%</t>
+        </is>
+      </c>
+      <c r="H592" s="25" t="inlineStr">
+        <is>
+          <t>1. 创建一笔订单：实付金额50元，投入成本50元。
+2. 支付完成后查看分佣明细</t>
+        </is>
+      </c>
+      <c r="I592" s="25" t="inlineStr">
+        <is>
+          <t>1. 利润=50-50=0元。
+2. 平台佣金=0×50%=0.00元。
+3. 代理商佣金=0×50%=0.00元。
+4. 一级分销员佣金=0×10%=0.00元。
+5. 所有角色佣金均为0.00元，分佣记录正常生成但金额为0</t>
+        </is>
+      </c>
+      <c r="J592" s="25" t="inlineStr">
+        <is>
+          <t>需求4.5.8分佣边界：利润为0所有人佣金为0</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="8" t="inlineStr">
+        <is>
+          <t>管理后台</t>
+        </is>
+      </c>
+      <c r="B593" s="8" t="inlineStr"/>
+      <c r="C593" s="8" t="inlineStr">
+        <is>
+          <t>fyxt-bl-002</t>
+        </is>
+      </c>
+      <c r="D593" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E593" s="8" t="n"/>
+      <c r="F593" s="8" t="inlineStr">
+        <is>
+          <t>验证利润为负（投入&gt;实付）时后端校验拦截</t>
+        </is>
+      </c>
+      <c r="G593" s="8" t="inlineStr">
+        <is>
+          <t>1. 管理后台已登录</t>
+        </is>
+      </c>
+      <c r="H593" s="8" t="inlineStr">
+        <is>
+          <t>1. 尝试在后台创建/配置一个商品：售价30元，成本50元。
+2. 保存商品配置。
+3. 如果保存成功，用户下单该商品后查看分佣</t>
+        </is>
+      </c>
+      <c r="I593" s="8" t="inlineStr">
+        <is>
+          <t>1. 后端校验拦截：提示"售价不能低于成本"或"利润不能为负"。
+2. 不允许保存该配置。
+3. 如果系统允许（异常情况），分佣计算不应产生负数佣金</t>
+        </is>
+      </c>
+      <c r="J593" s="8" t="inlineStr">
+        <is>
+          <t>需求4.5.8：利润为负不应出现，需后端校验拦截</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J453"/>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="E67:E90"/>
     <mergeCell ref="A552:J552"/>
+    <mergeCell ref="A584:J584"/>
     <mergeCell ref="E20:E37"/>
     <mergeCell ref="E38:E56"/>
     <mergeCell ref="A582:J582"/>
@@ -27291,7 +27751,7 @@
         </is>
       </c>
       <c r="C73" s="12" t="n">
-        <v>563</v>
+        <v>572</v>
       </c>
     </row>
     <row r="74">

</xml_diff>